<commit_message>
Complete placements report with Margin column for all 71 placements, sorted newest first
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018EeLbrdHRsMxxPUghfX52G
</commit_message>
<xml_diff>
--- a/placements_with_margin.xlsx
+++ b/placements_with_margin.xlsx
@@ -39,7 +39,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -49,11 +49,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00305496"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -69,14 +64,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -1961,7 +1955,9 @@
           <t>Indeed</t>
         </is>
       </c>
-      <c r="K29" s="4" t="n"/>
+      <c r="K29" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2012,7 +2008,9 @@
           <t>Indeed</t>
         </is>
       </c>
-      <c r="K30" s="4" t="n"/>
+      <c r="K30" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2063,7 +2061,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K31" s="4" t="n"/>
+      <c r="K31" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2163,7 +2163,9 @@
           <t>Indeed</t>
         </is>
       </c>
-      <c r="K33" s="4" t="n"/>
+      <c r="K33" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2267,7 +2269,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K35" s="4" t="n"/>
+      <c r="K35" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2371,7 +2375,9 @@
           <t>Linkedin Job Post</t>
         </is>
       </c>
-      <c r="K37" s="4" t="n"/>
+      <c r="K37" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2422,7 +2428,9 @@
           <t>Indeed</t>
         </is>
       </c>
-      <c r="K38" s="4" t="n"/>
+      <c r="K38" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2473,7 +2481,9 @@
           <t>Indeed</t>
         </is>
       </c>
-      <c r="K39" s="4" t="n"/>
+      <c r="K39" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2630,7 +2640,9 @@
           <t>Dice</t>
         </is>
       </c>
-      <c r="K42" s="4" t="n"/>
+      <c r="K42" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -2677,7 +2689,9 @@
           <t>Indeed</t>
         </is>
       </c>
-      <c r="K43" s="4" t="n"/>
+      <c r="K43" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2777,7 +2791,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K45" s="4" t="n"/>
+      <c r="K45" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2828,7 +2844,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K46" s="4" t="n"/>
+      <c r="K46" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2879,7 +2897,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K47" s="4" t="n"/>
+      <c r="K47" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -3036,7 +3056,9 @@
           <t>Indeed</t>
         </is>
       </c>
-      <c r="K50" s="4" t="n"/>
+      <c r="K50" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -3087,7 +3109,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K51" s="4" t="n"/>
+      <c r="K51" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -3138,7 +3162,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K52" s="4" t="n"/>
+      <c r="K52" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -3185,7 +3211,9 @@
           <t>LinkedIn Job Post</t>
         </is>
       </c>
-      <c r="K53" s="4" t="n"/>
+      <c r="K53" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -3236,7 +3264,9 @@
           <t>Linkedin</t>
         </is>
       </c>
-      <c r="K54" s="4" t="n"/>
+      <c r="K54" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -3283,7 +3313,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K55" s="4" t="n"/>
+      <c r="K55" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -3334,7 +3366,9 @@
           <t>Dice</t>
         </is>
       </c>
-      <c r="K56" s="4" t="n"/>
+      <c r="K56" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -3434,7 +3468,9 @@
           <t>Indeed</t>
         </is>
       </c>
-      <c r="K58" s="4" t="n"/>
+      <c r="K58" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -3485,7 +3521,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K59" s="4" t="n"/>
+      <c r="K59" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -3532,7 +3570,9 @@
           <t>Indeed Job Post</t>
         </is>
       </c>
-      <c r="K60" s="4" t="n"/>
+      <c r="K60" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -3583,7 +3623,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K61" s="4" t="n"/>
+      <c r="K61" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -3634,7 +3676,9 @@
           <t>Dice</t>
         </is>
       </c>
-      <c r="K62" s="4" t="n"/>
+      <c r="K62" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -3685,7 +3729,9 @@
           <t>Linkedin</t>
         </is>
       </c>
-      <c r="K63" s="4" t="n"/>
+      <c r="K63" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -3736,7 +3782,9 @@
           <t>Referral</t>
         </is>
       </c>
-      <c r="K64" s="4" t="n"/>
+      <c r="K64" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -3783,7 +3831,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K65" s="4" t="n"/>
+      <c r="K65" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -3830,7 +3880,9 @@
           <t>Linkedin</t>
         </is>
       </c>
-      <c r="K66" s="4" t="n"/>
+      <c r="K66" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -3930,7 +3982,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K68" s="4" t="n"/>
+      <c r="K68" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -3981,7 +4035,9 @@
           <t>Indeed</t>
         </is>
       </c>
-      <c r="K69" s="4" t="n"/>
+      <c r="K69" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -4032,7 +4088,9 @@
           <t>Indeed</t>
         </is>
       </c>
-      <c r="K70" s="4" t="n"/>
+      <c r="K70" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -4079,7 +4137,9 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K71" s="4" t="n"/>
+      <c r="K71" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -4135,12 +4195,12 @@
       </c>
     </row>
     <row r="73">
-      <c r="J73" s="5" t="inlineStr">
+      <c r="J73" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="K73" s="6">
+      <c r="K73" s="5">
         <f>SUM(K2:K72)</f>
         <v/>
       </c>

</xml_diff>